<commit_message>
Create health insurance PDF recovery module
</commit_message>
<xml_diff>
--- a/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/health_insurance_unreadable_files.xlsx
+++ b/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/health_insurance_unreadable_files.xlsx
@@ -81,6 +81,26 @@
           <t>recommended_fix</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>recovery_status</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>recovery_method</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>recovered_text_path</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>extracted_text_length</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -153,6 +173,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -225,6 +265,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -297,6 +357,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -369,6 +449,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -441,6 +541,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -513,6 +633,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -585,6 +725,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -657,6 +817,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -729,6 +909,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -801,6 +1001,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -873,6 +1093,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -945,6 +1185,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1017,6 +1277,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1089,6 +1369,26 @@
           <t>Install cryptography/pdfplumber/pymupdf or export an unlocked PDF, then rerun extraction.</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1161,6 +1461,26 @@
           <t>Install cryptography/pdfplumber/pymupdf or export an unlocked PDF, then rerun extraction.</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1233,6 +1553,26 @@
           <t>Install cryptography/pdfplumber/pymupdf or export an unlocked PDF, then rerun extraction.</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1305,6 +1645,26 @@
           <t>Install cryptography/pdfplumber/pymupdf or export an unlocked PDF, then rerun extraction.</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1377,6 +1737,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1449,6 +1829,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1521,6 +1921,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1593,6 +2013,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1665,6 +2105,26 @@
           <t>Install cryptography/pdfplumber/pymupdf or export an unlocked PDF, then rerun extraction.</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1737,6 +2197,26 @@
           <t>Install cryptography/pdfplumber/pymupdf or export an unlocked PDF, then rerun extraction.</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1809,6 +2289,26 @@
           <t>Install cryptography/pdfplumber/pymupdf or export an unlocked PDF, then rerun extraction.</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1881,6 +2381,26 @@
           <t>Install cryptography/pdfplumber/pymupdf or export an unlocked PDF, then rerun extraction.</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1953,6 +2473,26 @@
           <t>Install cryptography/pdfplumber/pymupdf or export an unlocked PDF, then rerun extraction.</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2025,6 +2565,26 @@
           <t>Run OCR or provide a text-based/exported PDF.</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>image OCR required</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2095,6 +2655,26 @@
       <c r="N29" t="inlineStr">
         <is>
           <t>Run OCR or provide a text-based/exported PDF.</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>OCR_REQUIRED after PyMuPDF/pypdf/pdfplumber attempts</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>

</xml_diff>